<commit_message>
chat module has been updated
</commit_message>
<xml_diff>
--- a/attendance/python-script/all_users.xlsx
+++ b/attendance/python-script/all_users.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C1363"/>
+  <dimension ref="A1:C1373"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -23587,6 +23587,176 @@
         </is>
       </c>
     </row>
+    <row r="1364">
+      <c r="A1364" t="inlineStr">
+        <is>
+          <t>1363</t>
+        </is>
+      </c>
+      <c r="B1364" t="inlineStr">
+        <is>
+          <t>Stephen</t>
+        </is>
+      </c>
+      <c r="C1364" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+    </row>
+    <row r="1365">
+      <c r="A1365" t="inlineStr">
+        <is>
+          <t>1364</t>
+        </is>
+      </c>
+      <c r="B1365" t="inlineStr">
+        <is>
+          <t>Abdullah</t>
+        </is>
+      </c>
+      <c r="C1365" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+    </row>
+    <row r="1366">
+      <c r="A1366" t="inlineStr">
+        <is>
+          <t>1365</t>
+        </is>
+      </c>
+      <c r="B1366" t="inlineStr">
+        <is>
+          <t>Arslan</t>
+        </is>
+      </c>
+      <c r="C1366" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+    </row>
+    <row r="1367">
+      <c r="A1367" t="inlineStr">
+        <is>
+          <t>1366</t>
+        </is>
+      </c>
+      <c r="B1367" t="inlineStr">
+        <is>
+          <t>Rahul</t>
+        </is>
+      </c>
+      <c r="C1367" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+    </row>
+    <row r="1368">
+      <c r="A1368" t="inlineStr">
+        <is>
+          <t>1367</t>
+        </is>
+      </c>
+      <c r="B1368" t="inlineStr">
+        <is>
+          <t>Asim</t>
+        </is>
+      </c>
+      <c r="C1368" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+    </row>
+    <row r="1369">
+      <c r="A1369" t="inlineStr">
+        <is>
+          <t>1368</t>
+        </is>
+      </c>
+      <c r="B1369" t="inlineStr">
+        <is>
+          <t>Shoaib</t>
+        </is>
+      </c>
+      <c r="C1369" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+    </row>
+    <row r="1370">
+      <c r="A1370" t="inlineStr">
+        <is>
+          <t>1369</t>
+        </is>
+      </c>
+      <c r="B1370" t="inlineStr">
+        <is>
+          <t>Mubashir</t>
+        </is>
+      </c>
+      <c r="C1370" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+    </row>
+    <row r="1371">
+      <c r="A1371" t="inlineStr">
+        <is>
+          <t>1370</t>
+        </is>
+      </c>
+      <c r="B1371" t="inlineStr">
+        <is>
+          <t>Numan</t>
+        </is>
+      </c>
+      <c r="C1371" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+    </row>
+    <row r="1372">
+      <c r="A1372" t="inlineStr">
+        <is>
+          <t>1371</t>
+        </is>
+      </c>
+      <c r="B1372" t="inlineStr">
+        <is>
+          <t>Sadaf</t>
+        </is>
+      </c>
+      <c r="C1372" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+    </row>
+    <row r="1373">
+      <c r="A1373" t="inlineStr">
+        <is>
+          <t>1372</t>
+        </is>
+      </c>
+      <c r="B1373" t="inlineStr">
+        <is>
+          <t>Noor</t>
+        </is>
+      </c>
+      <c r="C1373" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>